<commit_message>
All Edits are done
</commit_message>
<xml_diff>
--- a/data/OWNER.xlsx
+++ b/data/OWNER.xlsx
@@ -47,9 +47,6 @@
     <t>Emirates ID No</t>
   </si>
   <si>
-    <t>Date Of Bairh</t>
-  </si>
-  <si>
     <t>Mobile Number</t>
   </si>
   <si>
@@ -177,6 +174,9 @@
   </si>
   <si>
     <t>025152141521</t>
+  </si>
+  <si>
+    <t>Date Of Birh</t>
   </si>
 </sst>
 </file>
@@ -558,7 +558,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -593,7 +593,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>3</v>
@@ -602,465 +602,465 @@
         <v>4</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:15">
       <c r="A2" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
         <v>14</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
       </c>
       <c r="D2">
         <v>125</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G2" s="4">
         <v>31103</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I2">
         <v>6352411</v>
       </c>
       <c r="J2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L2" t="s">
+        <v>17</v>
+      </c>
+      <c r="M2" t="s">
+        <v>17</v>
+      </c>
+      <c r="N2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="M2" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" t="s">
         <v>19</v>
-      </c>
-      <c r="O2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
         <v>21</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
       </c>
       <c r="D3">
         <v>119</v>
       </c>
       <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="G3" s="4">
         <v>27404</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I3">
         <v>695111</v>
       </c>
       <c r="J3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M3" t="s">
-        <v>27</v>
-      </c>
-      <c r="N3" s="3" t="s">
+      <c r="O3" t="s">
         <v>28</v>
-      </c>
-      <c r="O3" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="A4" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
         <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
       </c>
       <c r="D4">
         <v>125</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G4" s="4">
         <v>31103</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I4">
         <v>6354121</v>
       </c>
       <c r="J4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M4" t="s">
+        <v>17</v>
+      </c>
+      <c r="N4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="M4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N4" s="3" t="s">
+      <c r="O4" t="s">
         <v>19</v>
-      </c>
-      <c r="O4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
       </c>
       <c r="D5">
         <v>119</v>
       </c>
       <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="G5" s="4">
         <v>27404</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I5">
         <v>6911411</v>
       </c>
       <c r="J5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L5" t="s">
+        <v>26</v>
+      </c>
+      <c r="M5" t="s">
+        <v>26</v>
+      </c>
+      <c r="N5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M5" t="s">
-        <v>27</v>
-      </c>
-      <c r="N5" s="3" t="s">
+      <c r="O5" t="s">
         <v>28</v>
-      </c>
-      <c r="O5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:15">
       <c r="A6" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
         <v>14</v>
-      </c>
-      <c r="C6" t="s">
-        <v>15</v>
       </c>
       <c r="D6">
         <v>125</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G6" s="4">
         <v>31103</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I6">
         <v>6352421</v>
       </c>
       <c r="J6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L6" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="M6" t="s">
-        <v>18</v>
-      </c>
-      <c r="N6" s="3" t="s">
+      <c r="O6" t="s">
         <v>19</v>
-      </c>
-      <c r="O6" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
         <v>21</v>
-      </c>
-      <c r="C7" t="s">
-        <v>22</v>
       </c>
       <c r="D7">
         <v>119</v>
       </c>
       <c r="E7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="G7" s="4">
         <v>27404</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I7">
         <v>6951111</v>
       </c>
       <c r="J7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L7" t="s">
+        <v>26</v>
+      </c>
+      <c r="M7" t="s">
+        <v>26</v>
+      </c>
+      <c r="N7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M7" t="s">
-        <v>27</v>
-      </c>
-      <c r="N7" s="3" t="s">
+      <c r="O7" t="s">
         <v>28</v>
-      </c>
-      <c r="O7" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:15">
       <c r="A8" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
         <v>14</v>
-      </c>
-      <c r="C8" t="s">
-        <v>15</v>
       </c>
       <c r="D8">
         <v>125</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G8" s="4">
         <v>31103</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I8">
         <v>6524121</v>
       </c>
       <c r="J8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L8" t="s">
+        <v>17</v>
+      </c>
+      <c r="M8" t="s">
+        <v>17</v>
+      </c>
+      <c r="N8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="M8" t="s">
-        <v>18</v>
-      </c>
-      <c r="N8" s="3" t="s">
+      <c r="O8" t="s">
         <v>19</v>
-      </c>
-      <c r="O8" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:15">
       <c r="A9" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
         <v>21</v>
-      </c>
-      <c r="C9" t="s">
-        <v>22</v>
       </c>
       <c r="D9">
         <v>119</v>
       </c>
       <c r="E9" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="G9" s="4">
         <v>27404</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="I9">
         <v>6951411</v>
       </c>
       <c r="J9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L9" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" t="s">
+        <v>26</v>
+      </c>
+      <c r="N9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="M9" t="s">
-        <v>27</v>
-      </c>
-      <c r="N9" s="3" t="s">
+      <c r="O9" t="s">
         <v>28</v>
-      </c>
-      <c r="O9" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
         <v>14</v>
-      </c>
-      <c r="C10" t="s">
-        <v>15</v>
       </c>
       <c r="D10">
         <v>125</v>
       </c>
       <c r="E10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G10" s="4">
         <v>31103</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I10">
         <v>6324121</v>
       </c>
       <c r="J10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L10" t="s">
+        <v>17</v>
+      </c>
+      <c r="M10" t="s">
+        <v>17</v>
+      </c>
+      <c r="N10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="M10" t="s">
-        <v>18</v>
-      </c>
-      <c r="N10" s="3" t="s">
+      <c r="O10" t="s">
         <v>19</v>
-      </c>
-      <c r="O10" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:15">
       <c r="A11" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
         <v>33</v>
-      </c>
-      <c r="C11" t="s">
-        <v>34</v>
       </c>
       <c r="D11">
         <v>125</v>
       </c>
       <c r="E11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G11" s="4">
         <v>34213</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I11">
         <v>632421</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:15">

</xml_diff>